<commit_message>
going to send out
</commit_message>
<xml_diff>
--- a/BOOST_package/BOOST_BOM.xlsx
+++ b/BOOST_package/BOOST_BOM.xlsx
@@ -218,7 +218,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">COST_SUMMARY.md gives $600.61</t>
+          <t xml:space="preserve">COST_SUMMARY.md gives $599.01</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R14</t>
+          <t xml:space="preserve">R15</t>
         </is>
       </c>
       <c r="C24" s="10">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 1M ohm 1 % (0805)</t>
+          <t xml:space="preserve">resistor 10 ohm 1 % (0805)</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
@@ -2292,12 +2292,12 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805W8F1004T5E</t>
+          <t xml:space="preserve">0805W8F100JT5E</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17514</t>
+          <t xml:space="preserve">C17415</t>
         </is>
       </c>
       <c r="I24" s="0" t="inlineStr">
@@ -2306,13 +2306,13 @@
         </is>
       </c>
       <c r="J24" s="3">
-        <v>0.0043</v>
+        <v>0.004</v>
       </c>
       <c r="K24" s="2">
         <f>D24*J24</f>
       </c>
       <c r="L24" s="10">
-        <v>2420510</v>
+        <v>6880485</v>
       </c>
       <c r="M24" s="0" t="inlineStr">
         <is>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="N24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">top</t>
+          <t xml:space="preserve">bottom</t>
         </is>
       </c>
       <c r="O24" s="0" t="inlineStr">
@@ -2330,27 +2330,27 @@
         </is>
       </c>
       <c r="P24" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/18202-0805W8F1004T5E/C17514","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/18103-0805W8F100JT5E/C17415","JLC")</f>
       </c>
       <c r="Q24" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f1004t5e_C17514.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f100jt5e_C17415.html","LCSC")</f>
       </c>
       <c r="R24" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010200_UNI-ROYAL-Uniroyal-Elec-0805W8F1004T5E_C17514.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010216_UNI-ROYAL-Uniroyal-Elec-0805W8F100JT5E_C17415.pdf","PDF")</f>
       </c>
       <c r="S24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1M</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 125mW 150V 1MΩ Thick Film Resistor ±1% ±100ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">-55℃~+155℃ 10Ω 125mW 150V Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="U24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">value and package from the schematic; 1% thick film, JLC Basic where one exists; on LX (65 V peak): 150 V rated</t>
+          <t xml:space="preserve">value and package from the schematic; 1% thick film, JLC Basic where one exists</t>
         </is>
       </c>
     </row>
@@ -2360,18 +2360,18 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R15</t>
+          <t xml:space="preserve">R21 R48 R60 R72</t>
         </is>
       </c>
       <c r="C25" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" s="10">
         <f>C25*2+20</f>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 10 ohm 1 % (0805)</t>
+          <t xml:space="preserve">resistor 5.1 ohm 1 % (0805)</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
@@ -2381,12 +2381,12 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805W8F100JT5E</t>
+          <t xml:space="preserve">0805W8F510KT5E</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17415</t>
+          <t xml:space="preserve">C17724</t>
         </is>
       </c>
       <c r="I25" s="0" t="inlineStr">
@@ -2395,13 +2395,13 @@
         </is>
       </c>
       <c r="J25" s="3">
-        <v>0.004</v>
+        <v>0.0041</v>
       </c>
       <c r="K25" s="2">
         <f>D25*J25</f>
       </c>
       <c r="L25" s="10">
-        <v>6880485</v>
+        <v>418343</v>
       </c>
       <c r="M25" s="0" t="inlineStr">
         <is>
@@ -2419,27 +2419,27 @@
         </is>
       </c>
       <c r="P25" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/18103-0805W8F100JT5E/C17415","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/18412-0805W8F510KT5E/C17724","JLC")</f>
       </c>
       <c r="Q25" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f100jt5e_C17415.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f510kt5e_C17724.html","LCSC")</f>
       </c>
       <c r="R25" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010216_UNI-ROYAL-Uniroyal-Elec-0805W8F100JT5E_C17415.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010200_UNI-ROYAL-Uniroyal-Elec-0805W8F510KT5E_C17724.pdf","PDF")</f>
       </c>
       <c r="S25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">5.1</t>
         </is>
       </c>
       <c r="T25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 10Ω 125mW 150V Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">-55℃~+155℃ 125mW 150V 5.1Ω Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="U25" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">value and package from the schematic; 1% thick film, JLC Basic where one exists</t>
+          <t xml:space="preserve">your choice of 2026-09-24; rev6: 5 -&gt; 5.1 Ohm (5.0 Ohm 0805 is not stocked), the value R59/R70 already use Alternates: C25273 4.99 Ohm</t>
         </is>
       </c>
     </row>
@@ -2449,18 +2449,18 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R21 R48 R60 R72</t>
+          <t xml:space="preserve">R22 R50 R56</t>
         </is>
       </c>
       <c r="C26" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" s="10">
         <f>C26*2+20</f>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 5.1 ohm 1 % (0805)</t>
+          <t xml:space="preserve">resistor 100 ohm 1 % (0603)</t>
         </is>
       </c>
       <c r="F26" s="0" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805W8F510KT5E</t>
+          <t xml:space="preserve">0603WAF1000T5E</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17724</t>
+          <t xml:space="preserve">C22775</t>
         </is>
       </c>
       <c r="I26" s="0" t="inlineStr">
@@ -2484,22 +2484,22 @@
         </is>
       </c>
       <c r="J26" s="3">
-        <v>0.0041</v>
+        <v>0.0031</v>
       </c>
       <c r="K26" s="2">
         <f>D26*J26</f>
       </c>
       <c r="L26" s="10">
-        <v>418343</v>
+        <v>11576722</v>
       </c>
       <c r="M26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805</t>
+          <t xml:space="preserve">0603</t>
         </is>
       </c>
       <c r="N26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bottom</t>
+          <t xml:space="preserve">top</t>
         </is>
       </c>
       <c r="O26" s="0" t="inlineStr">
@@ -2508,27 +2508,27 @@
         </is>
       </c>
       <c r="P26" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/18412-0805W8F510KT5E/C17724","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/23502-0603WAF1000T5E/C22775","JLC")</f>
       </c>
       <c r="Q26" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f510kt5e_C17724.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0603waf1000t5e_C22775.html","LCSC")</f>
       </c>
       <c r="R26" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010200_UNI-ROYAL-Uniroyal-Elec-0805W8F510KT5E_C17724.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2411221126_UNI-ROYAL-Uniroyal-Elec-0603WAF1000T5E_C22775.pdf","PDF")</f>
       </c>
       <c r="S26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.1</t>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 125mW 150V 5.1Ω Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">-55℃~+155℃ 100mW 100Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="U26" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">your choice of 2026-09-24; rev6: 5 -&gt; 5.1 Ohm (5.0 Ohm 0805 is not stocked), the value R59/R70 already use Alternates: C25273 4.99 Ohm</t>
+          <t xml:space="preserve">value and package from the schematic; 1% thick film, JLC Basic where one exists</t>
         </is>
       </c>
     </row>
@@ -2538,18 +2538,18 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R22 R50 R56</t>
+          <t xml:space="preserve">R49 R61 R62 R73 R74 R75 R76 R104</t>
         </is>
       </c>
       <c r="C27" s="10">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D27" s="10">
         <f>C27*2+20</f>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 100 ohm 1 % (0603)</t>
+          <t xml:space="preserve">resistor 10k ohm 1 % (0603)</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
@@ -2559,12 +2559,12 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0603WAF1000T5E</t>
+          <t xml:space="preserve">0603WAF1002T5E</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C22775</t>
+          <t xml:space="preserve">C25804</t>
         </is>
       </c>
       <c r="I27" s="0" t="inlineStr">
@@ -2573,13 +2573,13 @@
         </is>
       </c>
       <c r="J27" s="3">
-        <v>0.0031</v>
+        <v>0.0018</v>
       </c>
       <c r="K27" s="2">
         <f>D27*J27</f>
       </c>
       <c r="L27" s="10">
-        <v>11576722</v>
+        <v>23109251</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="N27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">top</t>
+          <t xml:space="preserve">bottom/top</t>
         </is>
       </c>
       <c r="O27" s="0" t="inlineStr">
@@ -2597,22 +2597,22 @@
         </is>
       </c>
       <c r="P27" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/23502-0603WAF1000T5E/C22775","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/26547-0603WAF1002T5E/C25804","JLC")</f>
       </c>
       <c r="Q27" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0603waf1000t5e_C22775.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0603waf1002t5e_C25804.html","LCSC")</f>
       </c>
       <c r="R27" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2411221126_UNI-ROYAL-Uniroyal-Elec-0603WAF1000T5E_C22775.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010045_UNI-ROYAL-Uniroyal-Elec-0603WAF1002T5E_C25804.pdf","PDF")</f>
       </c>
       <c r="S27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">100</t>
+          <t xml:space="preserve">10k</t>
         </is>
       </c>
       <c r="T27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 100mW 100Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">-55℃~+155℃ 100mW 10kΩ 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="U27" s="11" t="inlineStr">
@@ -2627,18 +2627,18 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R49 R61 R62 R73 R74 R75 R76 R104</t>
+          <t xml:space="preserve">R59 R70</t>
         </is>
       </c>
       <c r="C28" s="10">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D28" s="10">
-        <f>C28*2+20</f>
+        <f>C28*2+0</f>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 10k ohm 1 % (0603)</t>
+          <t xml:space="preserve">resistor 5.1 ohm 1 % (0805)</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
@@ -2648,12 +2648,12 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0603WAF1002T5E</t>
+          <t xml:space="preserve">0805W8F510KT5E</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C25804</t>
+          <t xml:space="preserve">C17724</t>
         </is>
       </c>
       <c r="I28" s="0" t="inlineStr">
@@ -2662,17 +2662,17 @@
         </is>
       </c>
       <c r="J28" s="3">
-        <v>0.0018</v>
+        <v>0.0041</v>
       </c>
       <c r="K28" s="2">
         <f>D28*J28</f>
       </c>
       <c r="L28" s="10">
-        <v>23109251</v>
+        <v>418343</v>
       </c>
       <c r="M28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0603</t>
+          <t xml:space="preserve">0805</t>
         </is>
       </c>
       <c r="N28" s="0" t="inlineStr">
@@ -2686,22 +2686,22 @@
         </is>
       </c>
       <c r="P28" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/26547-0603WAF1002T5E/C25804","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/18412-0805W8F510KT5E/C17724","JLC")</f>
       </c>
       <c r="Q28" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0603waf1002t5e_C25804.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f510kt5e_C17724.html","LCSC")</f>
       </c>
       <c r="R28" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010045_UNI-ROYAL-Uniroyal-Elec-0603WAF1002T5E_C25804.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010200_UNI-ROYAL-Uniroyal-Elec-0805W8F510KT5E_C17724.pdf","PDF")</f>
       </c>
       <c r="S28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">10k</t>
+          <t xml:space="preserve">5.1</t>
         </is>
       </c>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 100mW 10kΩ 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">-55℃~+155℃ 125mW 150V 5.1Ω Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="U28" s="11" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R59 R70</t>
+          <t xml:space="preserve">U1 U17</t>
         </is>
       </c>
       <c r="C29" s="10">
@@ -2727,46 +2727,46 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">resistor 5.1 ohm 1 % (0805)</t>
+          <t xml:space="preserve">linear regulator 5 V 100 mA</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNI-ROYAL(Uniroyal Elec)</t>
+          <t xml:space="preserve">STMicroelectronics</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805W8F510KT5E</t>
+          <t xml:space="preserve">L78L05ACUTR</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17724</t>
+          <t xml:space="preserve">C43116</t>
         </is>
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basic</t>
+          <t xml:space="preserve">Extended</t>
         </is>
       </c>
       <c r="J29" s="3">
-        <v>0.0041</v>
+        <v>0.102</v>
       </c>
       <c r="K29" s="2">
         <f>D29*J29</f>
       </c>
       <c r="L29" s="10">
-        <v>418343</v>
+        <v>21384</v>
       </c>
       <c r="M29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805</t>
+          <t xml:space="preserve">SOT-89</t>
         </is>
       </c>
       <c r="N29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bottom/top</t>
+          <t xml:space="preserve">top</t>
         </is>
       </c>
       <c r="O29" s="0" t="inlineStr">
@@ -2775,27 +2775,27 @@
         </is>
       </c>
       <c r="P29" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/18412-0805W8F510KT5E/C17724","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/STMicroelectronics-L78L05ACUTR/C43116","JLC")</f>
       </c>
       <c r="Q29" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/chip-resistor-surface-mount_uni-royal-uniroyal-elec-0805w8f510kt5e_C17724.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/voltage-regulators-linear-low-drop-out-ldo-regulators_stmicroelectronics-l78l05acutr_C43116.html","LCSC")</f>
       </c>
       <c r="R29" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2206010200_UNI-ROYAL-Uniroyal-Elec-0805W8F510KT5E_C17724.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_1809200029_STMicroelectronics-L78L05ACUTR_C43116.pdf","PDF")</f>
       </c>
       <c r="S29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.1</t>
+          <t xml:space="preserve">L78L05</t>
         </is>
       </c>
       <c r="T29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-55℃~+155℃ 125mW 150V 5.1Ω Thick Film Resistor ±1% ±200ppm/℃ 0805 Chip Resistor - Surface Mount ROHS</t>
+          <t xml:space="preserve">0℃~+125℃@(Tj) 1 1.7V 100mA 20V 40uV 49dB@(120Hz) 5V 6mA Fixed Over Current Protection、Over Temperature Protection、Short Circuit Protection Positive SOT-89-3 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
         </is>
       </c>
       <c r="U29" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">value and package from the schematic; 1% thick film, JLC Basic where one exists</t>
+          <t xml:space="preserve">the device named in the schematic or the notes; ST L78L05ACUTR (pinout OUT-GND-IN as the symbol)</t>
         </is>
       </c>
     </row>
@@ -2805,33 +2805,33 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1 U17</t>
+          <t xml:space="preserve">U6 U11 U12</t>
         </is>
       </c>
       <c r="C30" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D30" s="10">
-        <f>C30*2+0</f>
+        <f>C30*2+20</f>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">linear regulator 5 V 100 mA</t>
+          <t xml:space="preserve">op-amp, rail-to-rail, 1 MHz</t>
         </is>
       </c>
       <c r="F30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">STMicroelectronics</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">L78L05ACUTR</t>
+          <t xml:space="preserve">TLV9001IDBVR</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C43116</t>
+          <t xml:space="preserve">C398363</t>
         </is>
       </c>
       <c r="I30" s="0" t="inlineStr">
@@ -2840,17 +2840,17 @@
         </is>
       </c>
       <c r="J30" s="3">
-        <v>0.102</v>
+        <v>0.0979</v>
       </c>
       <c r="K30" s="2">
         <f>D30*J30</f>
       </c>
       <c r="L30" s="10">
-        <v>21384</v>
+        <v>48438</v>
       </c>
       <c r="M30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-89</t>
+          <t xml:space="preserve">SOT-23-5</t>
         </is>
       </c>
       <c r="N30" s="0" t="inlineStr">
@@ -2864,27 +2864,27 @@
         </is>
       </c>
       <c r="P30" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/STMicroelectronics-L78L05ACUTR/C43116","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-TLV9001IDBVR/C398363","JLC")</f>
       </c>
       <c r="Q30" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/voltage-regulators-linear-low-drop-out-ldo-regulators_stmicroelectronics-l78l05acutr_C43116.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/operational-amplifier_texas-instruments-tlv9001idbvr_C398363.html","LCSC")</f>
       </c>
       <c r="R30" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_1809200029_STMicroelectronics-L78L05ACUTR_C43116.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2410010130_Texas-Instruments-TLV9001IDBVR_C398363.pdf","PDF")</f>
       </c>
       <c r="S30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">L78L05</t>
+          <t xml:space="preserve">TLV9001</t>
         </is>
       </c>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0℃~+125℃@(Tj) 1 1.7V 100mA 20V 40uV 49dB@(120Hz) 5V 6mA Fixed Over Current Protection、Over Temperature Protection、Short Circuit Protection Positive SOT-89-3 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
+          <t xml:space="preserve">-2.75V~-900mV、900mV~2.75V -40℃~+125℃ 1 1.6mV 1.8V~5.5V 1MHz 2V/us 2pA 4.7nV/√Hz@1kHz 40mA 5pA 600nV/℃ 60uA 86dB Enable/shutdown function、EMI filtering/RF suppression Rail-to-Rail Input, Rail-to-Rail Output SOT-23-5 Operational Amplifier ROHS</t>
         </is>
       </c>
       <c r="U30" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">the device named in the schematic or the notes; ST L78L05ACUTR (pinout OUT-GND-IN as the symbol)</t>
+          <t xml:space="preserve">approved 2026-10-01: TI TLV9001IDBVR (the DBV part: pins 1 OUT, 2 V-, 3 IN+, 4 IN-, 5 V+, as the MCP6241; NOT the TLV9001U). 1 MHz, 2 V/us, 1.6 mV max offset. LTspice re-runs (30 ms, 25 % PWM, cold start) match the MCP6241 within 0.05 % Alternates: C49889 MCP6241T-E/OT (before 2026-10-01)</t>
         </is>
       </c>
     </row>
@@ -2894,18 +2894,18 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">U6 U11 U12</t>
+          <t xml:space="preserve">U8 U10 U15 U19</t>
         </is>
       </c>
       <c r="C31" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="10">
-        <f>C31*2+20</f>
+        <f>C31*2+0</f>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">op-amp, rail-to-rail, 1 MHz</t>
+          <t xml:space="preserve">isolated dual gate driver</t>
         </is>
       </c>
       <c r="F31" s="0" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLV9001IDBVR</t>
+          <t xml:space="preserve">UCC21520DWR</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C398363</t>
+          <t xml:space="preserve">C601651</t>
         </is>
       </c>
       <c r="I31" s="0" t="inlineStr">
@@ -2929,22 +2929,22 @@
         </is>
       </c>
       <c r="J31" s="3">
-        <v>0.0979</v>
+        <v>0.8893</v>
       </c>
       <c r="K31" s="2">
         <f>D31*J31</f>
       </c>
       <c r="L31" s="10">
-        <v>48438</v>
+        <v>17156</v>
       </c>
       <c r="M31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOT-23-5</t>
+          <t xml:space="preserve">SOIC-16W</t>
         </is>
       </c>
       <c r="N31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">top</t>
+          <t xml:space="preserve">bottom</t>
         </is>
       </c>
       <c r="O31" s="0" t="inlineStr">
@@ -2953,27 +2953,27 @@
         </is>
       </c>
       <c r="P31" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-TLV9001IDBVR/C398363","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-UCC21520DWR/C601651","JLC")</f>
       </c>
       <c r="Q31" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/operational-amplifier_texas-instruments-tlv9001idbvr_C398363.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/isolators-gate-drivers_texas-instruments-ucc21520dwr_C601651.html","LCSC")</f>
       </c>
       <c r="R31" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2410010130_Texas-Instruments-TLV9001IDBVR_C398363.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2006102223_Texas-Instruments-UCC21520DWR_C601651.pdf","PDF")</f>
       </c>
       <c r="S31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLV9001</t>
+          <t xml:space="preserve">UCC21520DW</t>
         </is>
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-2.75V~-900mV、900mV~2.75V -40℃~+125℃ 1 1.6mV 1.8V~5.5V 1MHz 2V/us 2pA 4.7nV/√Hz@1kHz 40mA 5pA 600nV/℃ 60uA 86dB Enable/shutdown function、EMI filtering/RF suppression Rail-to-Rail Input, Rail-to-Rail Output SOT-23-5 Operational Amplifier ROHS</t>
+          <t xml:space="preserve">-40℃~+150℃@(Tj) 0.8V~1.2V 1.2V~2V 125kV/us 2 3V~18V 45ns 45ns 4A 5700 6A 9.2V~25V MOSFET、IGBT SOIC-16-300mil Isolators - Gate Drivers ROHS</t>
         </is>
       </c>
       <c r="U31" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">approved 2026-10-01: TI TLV9001IDBVR (the DBV part: pins 1 OUT, 2 V-, 3 IN+, 4 IN-, 5 V+, as the MCP6241; NOT the TLV9001U). 1 MHz, 2 V/us, 1.6 mV max offset. LTspice re-runs (30 ms, 25 % PWM, cold start) match the MCP6241 within 0.05 % Alternates: C49889 MCP6241T-E/OT (before 2026-10-01)</t>
+          <t xml:space="preserve">the device named in the schematic or the notes</t>
         </is>
       </c>
     </row>
@@ -2983,33 +2983,33 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">U8 U10 U15 U19</t>
+          <t xml:space="preserve">U16</t>
         </is>
       </c>
       <c r="C32" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D32" s="10">
         <f>C32*2+0</f>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">isolated dual gate driver</t>
+          <t xml:space="preserve">linear regulator 12 V 1 A (7812)</t>
         </is>
       </c>
       <c r="F32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">UCC21520DWR</t>
+          <t xml:space="preserve">MC7812BD2TR4G</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C601651</t>
+          <t xml:space="preserve">C231294</t>
         </is>
       </c>
       <c r="I32" s="0" t="inlineStr">
@@ -3018,22 +3018,22 @@
         </is>
       </c>
       <c r="J32" s="3">
-        <v>0.8893</v>
+        <v>0.5316</v>
       </c>
       <c r="K32" s="2">
         <f>D32*J32</f>
       </c>
       <c r="L32" s="10">
-        <v>17156</v>
+        <v>2024</v>
       </c>
       <c r="M32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOIC-16W</t>
+          <t xml:space="preserve">TO-263-3</t>
         </is>
       </c>
       <c r="N32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bottom</t>
+          <t xml:space="preserve">top</t>
         </is>
       </c>
       <c r="O32" s="0" t="inlineStr">
@@ -3042,27 +3042,27 @@
         </is>
       </c>
       <c r="P32" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-UCC21520DWR/C601651","JLC")</f>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/onsemi-MC7812BD2TR4G/C231294","JLC")</f>
       </c>
       <c r="Q32" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/isolators-gate-drivers_texas-instruments-ucc21520dwr_C601651.html","LCSC")</f>
+        <f>HYPERLINK("https://www.lcsc.com/product-detail/voltage-regulators-linear-low-drop-out-ldo-regulators_onsemi-mc7812bd2tr4g_C231294.html","LCSC")</f>
       </c>
       <c r="R32" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2006102223_Texas-Instruments-UCC21520DWR_C601651.pdf","PDF")</f>
+        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2210210200_onsemi-MC7812BD2TR4G_C231294.pdf","PDF")</f>
       </c>
       <c r="S32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">UCC21520DW</t>
+          <t xml:space="preserve">MC7812</t>
         </is>
       </c>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+150℃@(Tj) 0.8V~1.2V 1.2V~2V 125kV/us 2 3V~18V 45ns 45ns 4A 5700 6A 9.2V~25V MOSFET、IGBT SOIC-16-300mil Isolators - Gate Drivers ROHS</t>
+          <t xml:space="preserve">-40℃~+125℃@(Tj) 1 12V 1A 27V 2V@(1.0A) 3.4mA 60dB@(120Hz) Fixed Over Temperature Protection、Short Circuit Protection Positive TO-263-2 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
         </is>
       </c>
       <c r="U32" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">the device named in the schematic or the notes</t>
+          <t xml:space="preserve">approved 2026-10-01: onsemi MC7812BD2TR4G. Its D2PAK (case 936) fits the TO-263-3 footprint: pins 1 IN and 3 OUT at 2.54 mm pitch, tab = pin 2 GND, the centre lead is cut (pad 2 stays empty, it is GND). 35 V in, -40 to +125 C. About 1.5 V dropout, so at the end of a 4S discharge the LEDs fade from about 12.7 V open-circuit (simulated: BOOST_split_boards/mc7812_lowbatt_2026-10-01) Alternates: C38744 MC7812CD2TR4G (0 to +125 C); C2877347 LM2940S-12/NOPB (before 2026-10-01)</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">U16</t>
+          <t xml:space="preserve">U25</t>
         </is>
       </c>
       <c r="C33" s="10">
@@ -3083,22 +3083,22 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">linear regulator 12 V 1 A (7812)</t>
+          <t xml:space="preserve">current-sense amplifier, gain 100</t>
         </is>
       </c>
       <c r="F33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">onsemi</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MC7812BD2TR4G</t>
+          <t xml:space="preserve">INA241A4IDR</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C231294</t>
+          <t xml:space="preserve">C22427873</t>
         </is>
       </c>
       <c r="I33" s="0" t="inlineStr">
@@ -3107,17 +3107,17 @@
         </is>
       </c>
       <c r="J33" s="3">
-        <v>0.5316</v>
+        <v>3.5277</v>
       </c>
       <c r="K33" s="2">
         <f>D33*J33</f>
       </c>
       <c r="L33" s="10">
-        <v>2024</v>
+        <v>116</v>
       </c>
       <c r="M33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TO-263-3</t>
+          <t xml:space="preserve">SOIC-8</t>
         </is>
       </c>
       <c r="N33" s="0" t="inlineStr">
@@ -3131,122 +3131,52 @@
         </is>
       </c>
       <c r="P33" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/onsemi-MC7812BD2TR4G/C231294","JLC")</f>
-      </c>
-      <c r="Q33" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/product-detail/voltage-regulators-linear-low-drop-out-ldo-regulators_onsemi-mc7812bd2tr4g_C231294.html","LCSC")</f>
-      </c>
-      <c r="R33" s="5">
-        <f>HYPERLINK("https://www.lcsc.com/datasheet/lcsc_datasheet_2210210200_onsemi-MC7812BD2TR4G_C231294.pdf","PDF")</f>
-      </c>
+        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-INA241A4IDR/C22427873","JLC")</f>
+      </c>
+      <c r="Q33" s="0"/>
+      <c r="R33" s="0"/>
       <c r="S33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">MC7812</t>
+          <t xml:space="preserve">INA241A4</t>
         </is>
       </c>
       <c r="T33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+125℃@(Tj) 1 12V 1A 27V 2V@(1.0A) 3.4mA 60dB@(120Hz) Fixed Over Temperature Protection、Short Circuit Protection Positive TO-263-2 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
+          <t xml:space="preserve">SOIC-8 Current Sense Amplifiers ROHS</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">approved 2026-10-01: onsemi MC7812BD2TR4G. Its D2PAK (case 936) fits the TO-263-3 footprint: pins 1 IN and 3 OUT at 2.54 mm pitch, tab = pin 2 GND, the centre lead is cut (pad 2 stays empty, it is GND). 35 V in, -40 to +125 C. About 1.5 V dropout, so at the end of a 4S discharge the LEDs fade from about 12.7 V open-circuit (simulated: BOOST_split_boards/mc7812_lowbatt_2026-10-01) Alternates: C38744 MC7812CD2TR4G (0 to +125 C); C2877347 LM2940S-12/NOPB (before 2026-10-01)</t>
+          <t xml:space="preserve">your choice of 2026-09-24; rev6: gain 100 V/V with the 1 mOhm R1; TI SBOSA30D: same SOIC-8 pinout for every gain, 1.1 MHz for all gains Alternates: C22427652 INA241A3IDR (rev5)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10">
-        <v>33</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U25</t>
-        </is>
-      </c>
-      <c r="C34" s="10">
-        <v>1</v>
-      </c>
-      <c r="D34" s="10">
-        <f>C34*2+0</f>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">current-sense amplifier, gain 100</t>
-        </is>
-      </c>
-      <c r="F34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Texas Instruments</t>
-        </is>
-      </c>
-      <c r="G34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INA241A4IDR</t>
-        </is>
-      </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C22427873</t>
-        </is>
-      </c>
-      <c r="I34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Extended</t>
-        </is>
-      </c>
-      <c r="J34" s="3">
-        <v>3.5277</v>
-      </c>
-      <c r="K34" s="2">
-        <f>D34*J34</f>
-      </c>
-      <c r="L34" s="10">
-        <v>116</v>
-      </c>
-      <c r="M34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOIC-8</t>
-        </is>
-      </c>
-      <c r="N34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">top</t>
-        </is>
-      </c>
-      <c r="O34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JLC</t>
-        </is>
-      </c>
-      <c r="P34" s="5">
-        <f>HYPERLINK("https://jlcpcb.com/partdetail/TexasInstruments-INA241A4IDR/C22427873","JLC")</f>
-      </c>
-      <c r="Q34" s="0"/>
-      <c r="R34" s="0"/>
-      <c r="S34" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INA241A4</t>
-        </is>
-      </c>
-      <c r="T34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SOIC-8 Current Sense Amplifiers ROHS</t>
-        </is>
-      </c>
-      <c r="U34" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">your choice of 2026-09-24; rev6: gain 100 V/V with the 1 mOhm R1; TI SBOSA30D: same SOIC-8 pinout for every gain, 1.1 MHz for all gains Alternates: C22427652 INA241A3IDR (rev5)</t>
-        </is>
-      </c>
-    </row>
+</row>
     <row r="35">
-</row>
+      <c r="A35" s="0"/>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parts total (JLC lines, 2 boards + attrition)</t>
+        </is>
+      </c>
+      <c r="C35" s="0"/>
+      <c r="D35" s="0"/>
+      <c r="E35" s="0"/>
+      <c r="F35" s="0"/>
+      <c r="G35" s="0"/>
+      <c r="H35" s="0"/>
+      <c r="I35" s="0"/>
+      <c r="J35" s="0"/>
+      <c r="K35" s="7">
+        <f>SUMIFS(K2:K33,O2:O33,"JLC")</f>
+      </c>
+    </row>
     <row r="36">
       <c r="A36" s="0"/>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parts total (JLC lines, 2 boards + attrition)</t>
+          <t xml:space="preserve">Parts you buy or own (priced lines)</t>
         </is>
       </c>
       <c r="C36" s="0"/>
@@ -3258,14 +3188,14 @@
       <c r="I36" s="0"/>
       <c r="J36" s="0"/>
       <c r="K36" s="7">
-        <f>SUMIFS(K2:K34,O2:O34,"JLC")</f>
+        <f>SUMIFS(K2:K33,O2:O33,"you (hand)")</f>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0"/>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parts you buy or own (priced lines)</t>
+          <t xml:space="preserve">Unique JLC part numbers (feeder loading $1.53 each)</t>
         </is>
       </c>
       <c r="C37" s="0"/>
@@ -3276,31 +3206,12 @@
       <c r="H37" s="0"/>
       <c r="I37" s="0"/>
       <c r="J37" s="0"/>
-      <c r="K37" s="7">
-        <f>SUMIFS(K2:K34,O2:O34,"you (hand)")</f>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="0"/>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unique JLC part numbers (feeder loading $1.53 each)</t>
-        </is>
-      </c>
-      <c r="C38" s="0"/>
-      <c r="D38" s="0"/>
-      <c r="E38" s="0"/>
-      <c r="F38" s="0"/>
-      <c r="G38" s="0"/>
-      <c r="H38" s="0"/>
-      <c r="I38" s="0"/>
-      <c r="J38" s="0"/>
-      <c r="K38" s="10">
-        <v>29</v>
+      <c r="K37" s="10">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U34"/>
+  <autoFilter ref="A1:U33"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
@@ -4583,11 +4494,11 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R2 R6 R31 R33 R39 R41 R67 R77 R83 R85 R99 R100 R101 R102 R103</t>
+          <t xml:space="preserve">R2 R6 R31 R33 R39 R41 R67 R77 R83 R85 R100 R101 R103</t>
         </is>
       </c>
       <c r="C15" s="10">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D15" s="10">
         <f>C15*2+20</f>
@@ -4761,11 +4672,11 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R4 R54 R55 R58 R71</t>
+          <t xml:space="preserve">R4 R54 R55 R58 R71 R99 R102</t>
         </is>
       </c>
       <c r="C17" s="10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17" s="10">
         <f>C17*2+20</f>
@@ -5473,11 +5384,11 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">R27 R37 R45</t>
+          <t xml:space="preserve">R27 R37 R45 R106 R107</t>
         </is>
       </c>
       <c r="C25" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D25" s="10">
         <f>C25*2+20</f>
@@ -7835,7 +7746,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>'Power board'!K38*1.53</f>
+        <f>'Power board'!K37*1.53</f>
       </c>
       <c r="C5" s="2">
         <f>'Control card'!K47*1.53</f>
@@ -7856,11 +7767,11 @@
         <v>0.91</v>
       </c>
       <c r="C6" s="2">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">570 / 944 joints for 2 boards</t>
+          <t xml:space="preserve">566 / 952 joints for 2 boards</t>
         </is>
       </c>
     </row>
@@ -7871,7 +7782,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>'Power board'!K36</f>
+        <f>'Power board'!K35</f>
       </c>
       <c r="C7" s="2">
         <f>'Control card'!K45</f>

</xml_diff>